<commit_message>
grupo 24/7 afinado con la sesión del 22-oct
</commit_message>
<xml_diff>
--- a/grupo-soporte-24-7.xlsx
+++ b/grupo-soporte-24-7.xlsx
@@ -101,9 +101,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -470,11 +468,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B18"/>
+  <dimension ref="B2:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="98" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -498,10 +496,10 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="34" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>El grupo de WhatsApp donde se reportan y se resuelven en el momento las fallas de tag en caseta durante el piloto. Atención 24/7.</t>
+          <t>El grupo de WhatsApp donde se reportan y se destraban en el momento las fallas de tag en caseta, los cruces rechazados y las incidencias operativas durante el piloto. Atención 24/7, incluidos fines de semana.</t>
         </is>
       </c>
     </row>
@@ -512,10 +510,10 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>• Equipo de soporte de Uvicuo.  • Mesa de monitoreo del proveedor de telepeaje (Televía), 24/7.  • De su operación: los jefes de patio (o quien pueda reportar la falla del tag de sus unidades). NO entran operadores: son administradores que nos reportan.</t>
+          <t>• Equipo de soporte de Uvicuo (Chema es el punto de contacto principal).  • Mesa de monitoreo del proveedor de telepeaje (Televía), 24/7.  • De su operación: los jefes de patio (o quien pueda reportar la falla del tag de sus unidades). NO entran operadores: son administradores que nos reportan.</t>
         </is>
       </c>
     </row>
@@ -526,36 +524,50 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="34" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Aquí NO se comparte información sensible del viaje ni de la ruta: no es un canal oficial, es solo para destrabar fallas de tag.</t>
+          <t>NO es un canal oficial. Aquí NO se comparte información sensible: ubicaciones, tramos carreteros ni horarios. Solo coordinación operativa puntual de tags y casetas.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>¿Qué necesitamos de ti?</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t>Si algo no se resuelve (escalación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Llena la lista de abajo (celdas amarillas) con quién debe estar en el grupo: nombre, rol y número de WhatsApp. Uvicuo crea el grupo en cuanto nos confirmes que la lista ya tiene a todos sus integrantes.</t>
+          <t>1) Primero, el grupo de soporte 24/7.  2) Luego, Chema (líder del proyecto en Uvicuo).  3) Por último, la dirección de Uvicuo.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>¿Qué necesitamos de ti?</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Llena la lista de abajo (celdas amarillas): nombre, rol y número de WhatsApp de quien debe estar en el grupo. Uvicuo crea el grupo en cuanto nos confirmes que la lista ya tiene a todos sus integrantes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
           <t>¿Cómo nos lo regresas?</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="4" t="inlineStr">
+    <row r="21" ht="34" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Responde a nuestro correo de avance diario con este archivo lleno.</t>
         </is>
@@ -575,10 +587,10 @@
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>